<commit_message>
Reposiciona cachês de execução para O QUE PEDIMOS + nota de data da Fernanda
Os tres cachês de execução (Badaró, Mickaela, Zambonini — R$300 cada) saem
do bloco O QUE TRAZEMOS e passam para O QUE PEDIMOS, como custo a cobrir
pelo UP. Essa é uma mudança de dado explicitamente pedida pelo usuario e
diverge do que a planilha original trazia (Zambonini estava marcado como
'sem cachê' / R$0,00) — registrada aqui para rastreabilidade.

Novos totais, planilha e deck sincronizados e recalculados:
- O que trazemos: R$ 16.113,00 -> R$ 15.513,00
- O que pedimos:  R$  2.230,00 -> R$  3.130,00 (+ obra cimática, [A CONFIRMAR])

Slide 16 (apoio institucional): nota do slot Chill Out marca o horário como
[A CONFIRMAR], condicionado a grade de shows da Fernanda Pistelli — a
participação dela já está confirmada, só o horário exato depende da grade.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BgqkYwRoJUMewo2gzAx5Wf
</commit_message>
<xml_diff>
--- a/entregaveis/PEGA_VISAO_x_UP19_PROVISIONAMENTO.xlsx
+++ b/entregaveis/PEGA_VISAO_x_UP19_PROVISIONAMENTO.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="80">
   <si>
     <t xml:space="preserve">PEGA VISÃO × UNIVERSO PARALELLO 19</t>
   </si>
@@ -61,54 +61,54 @@
     <t xml:space="preserve">Live painting — Badaró</t>
   </si>
   <si>
-    <t xml:space="preserve">Cachê de execução.</t>
+    <t xml:space="preserve">Pintura ao vivo durante o festival. Cachê solicitado ao UP — ver bloco O QUE PEDIMOS.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cerâmica Às Cegas — Mickaela</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vivência guiada de olhos vendados, dias 28, 29 e 30/12. Cachê solicitado ao UP — ver bloco O QUE PEDIMOS.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cobertura audiovisual — Zambonini</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Captação e produção de conteúdo documental do projeto no UP19. Cachê solicitado ao UP — ver bloco O QUE PEDIMOS.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipamento audiovisual próprio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kit profissional do diretor: câmera Sony A7IV (33MP), lentes Sigma 24-70 Art e 70-200 GM, lapela Hollyland Lark Max 2, tripé, iluminação (tubo LED Sokani 25W, LED portátil 40W) e flash Godox V1. Garante padrão profissional de captação das experiências do Pega Visão e sustenta o intercâmbio de material audiovisual proposto com a equipe oficial do UP.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">45,000 em equipamentos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qualidade técnica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trust in Dance — Fernanda Pistelli</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experiência de dança guiada de olhos vendados. Participação artística, sem custo ao festival.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sets de referência</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dois sets autorais de Luis (Ota Blind) enviados para apreciação da curadoria.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Passagens aéreas — equipe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ida e volta: Luis Otávio, André Zambonini e Luis Badaró. Cotação real em 27/07/2026, ida 26/12/2026 e volta 05/01/2027 — Cuiabá↔Salvador (Badaró e Zambonini, 2 pax): R$5.317,00. Brasília↔Salvador (Luis, 1 pax): R$2.266,00.</t>
   </si>
   <si>
     <t xml:space="preserve">Pega Visão</t>
   </si>
   <si>
-    <t xml:space="preserve">Cerâmica Às Cegas — Mickaela</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vivência guiada de olhos vendados, dias 28, 29 e 30/12. Cachê de execução.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cobertura audiovisual — Zambonini</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Captação e produção de conteúdo documental do projeto no UP19, sem cachê.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Equipamento audiovisual próprio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kit profissional do diretor: câmera Sony A7IV (33MP), lentes Sigma 24-70 Art e 70-200 GM, lapela Hollyland Lark Max 2, tripé, iluminação (tubo LED Sokani 25W, LED portátil 40W) e flash Godox V1. Garante padrão profissional de captação das experiências do Pega Visão e sustenta o intercâmbio de material audiovisual proposto com a equipe oficial do UP.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">45,000 em equipamentos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Qualidade técnica</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trust in Dance — Fernanda Pistelli</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experiência de dança guiada de olhos vendados. Participação artística, sem custo ao festival.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sets de referência</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dois sets autorais de Luis (Ota Blind) enviados para apreciação da curadoria.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Passagens aéreas — equipe</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ida e volta: Luis Otávio, André Zambonini e Luis Badaró. Cotação real em 27/07/2026, ida 26/12/2026 e volta 05/01/2027 — Cuiabá↔Salvador (Badaró e Zambonini, 2 pax): R$5.317,00. Brasília↔Salvador (Luis, 1 pax): R$2.266,00.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Translado Salvador ↔ Pratigi</t>
   </si>
   <si>
@@ -145,15 +145,33 @@
     <t xml:space="preserve">Natureza</t>
   </si>
   <si>
+    <t xml:space="preserve">Cachê — Live painting (Badaró)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cachê de execução do live painting durante o festival.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Custo a cobrir pelo UP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cachê — Cerâmica Às Cegas (Mickaela)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cachê de execução da vivência guiada, dias 28, 29 e 30/12.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cachê — Cobertura audiovisual (Zambonini)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cachê de execução da captação documental do projeto no UP19.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Materiais — Live painting Badaró</t>
   </si>
   <si>
     <t xml:space="preserve">Tinta acrílica, suporte MDF 220×180, embalagem e proteção para transporte.</t>
   </si>
   <si>
-    <t xml:space="preserve">Custo a cobrir pelo UP</t>
-  </si>
-  <si>
     <t xml:space="preserve">Produção — Nova obra tátil (Cimática)</t>
   </si>
   <si>
@@ -220,7 +238,7 @@
     <t xml:space="preserve">Slot — Chill Out</t>
   </si>
   <si>
-    <t xml:space="preserve">Set de Ota Blind no Chill Out, em horário próximo à experiência Trust in Dance.</t>
+    <t xml:space="preserve">Set de Ota Blind no Chill Out, em horário próximo à experiência Trust in Dance — horário exato [A CONFIRMAR], conforme grade de shows de Fernanda Pistelli.</t>
   </si>
   <si>
     <t xml:space="preserve">Slot — UP Club</t>
@@ -342,6 +360,14 @@
     </font>
     <font>
       <b val="true"/>
+      <sz val="9"/>
+      <color rgb="FF8A6B33"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="10.5"/>
       <color rgb="FF1A1A1A"/>
       <name val="Arial"/>
@@ -352,14 +378,6 @@
       <b val="true"/>
       <sz val="9"/>
       <color rgb="FF6E7A2A"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="9"/>
-      <color rgb="FF8A6B33"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -584,34 +602,34 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="15" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -636,12 +654,12 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="19" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -912,7 +930,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D45"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="31"/>
@@ -974,82 +992,82 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="12" t="n">
-        <v>300</v>
+      <c r="C7" s="12" t="s">
+        <v>9</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="14" t="n">
-        <v>300</v>
-      </c>
-      <c r="D8" s="15" t="s">
-        <v>13</v>
+      <c r="C8" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" s="12" t="n">
-        <v>0</v>
+      <c r="C9" s="12" t="s">
+        <v>9</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="C10" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="D10" s="14" t="s">
         <v>20</v>
-      </c>
-      <c r="D10" s="16" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="D11" s="18" t="s">
+      <c r="D11" s="13" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" s="7" t="s">
         <v>24</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>25</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>9</v>
@@ -1060,16 +1078,16 @@
     </row>
     <row r="13" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="C13" s="15" t="n">
+        <v>7583</v>
+      </c>
+      <c r="D13" s="16" t="s">
         <v>27</v>
-      </c>
-      <c r="C13" s="12" t="n">
-        <v>7583</v>
-      </c>
-      <c r="D13" s="13" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1079,11 +1097,11 @@
       <c r="B14" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="14" t="n">
+      <c r="C14" s="17" t="n">
         <v>930</v>
       </c>
-      <c r="D14" s="15" t="s">
-        <v>13</v>
+      <c r="D14" s="18" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1093,11 +1111,11 @@
       <c r="B15" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="12" t="n">
+      <c r="C15" s="15" t="n">
         <v>7000</v>
       </c>
-      <c r="D15" s="13" t="s">
-        <v>13</v>
+      <c r="D15" s="16" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1121,10 +1139,10 @@
       <c r="B17" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="C17" s="17" t="s">
+      <c r="C17" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="D17" s="18" t="s">
+      <c r="D17" s="13" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1136,7 +1154,7 @@
       <c r="B19" s="20"/>
       <c r="C19" s="21" t="n">
         <f aca="false">SUM(C6:C17)</f>
-        <v>16113</v>
+        <v>15513</v>
       </c>
       <c r="D19" s="22"/>
     </row>
@@ -1163,15 +1181,15 @@
         <v>39</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
         <v>40</v>
       </c>
       <c r="B23" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="C23" s="12" t="n">
-        <v>980</v>
+      <c r="C23" s="15" t="n">
+        <v>300</v>
       </c>
       <c r="D23" s="24" t="s">
         <v>42</v>
@@ -1184,22 +1202,22 @@
       <c r="B24" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="C24" s="25" t="s">
-        <v>45</v>
-      </c>
-      <c r="D24" s="26" t="s">
+      <c r="C24" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="D24" s="25" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="B25" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="C25" s="12" t="n">
-        <v>750</v>
+      <c r="C25" s="15" t="n">
+        <v>300</v>
       </c>
       <c r="D25" s="24" t="s">
         <v>42</v>
@@ -1207,86 +1225,98 @@
     </row>
     <row r="26" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B26" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="B26" s="7" t="s">
+      <c r="C26" s="17" t="n">
+        <v>980</v>
+      </c>
+      <c r="D26" s="25" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="C26" s="14" t="n">
+      <c r="B27" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="C27" s="26" t="s">
+        <v>51</v>
+      </c>
+      <c r="D27" s="24" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C28" s="17" t="n">
+        <v>750</v>
+      </c>
+      <c r="D28" s="25" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="B29" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="C29" s="15" t="n">
         <v>500</v>
       </c>
-      <c r="D26" s="26" t="s">
+      <c r="D29" s="24" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="28" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="20" t="s">
-        <v>50</v>
-      </c>
-      <c r="B28" s="20"/>
-      <c r="C28" s="27" t="n">
-        <f aca="false">SUM(C23:C26)</f>
-        <v>2230</v>
-      </c>
-      <c r="D28" s="22"/>
-    </row>
-    <row r="29" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="28" t="s">
-        <v>51</v>
-      </c>
-      <c r="B29" s="28"/>
-      <c r="C29" s="28"/>
-      <c r="D29" s="28"/>
-    </row>
-    <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="31" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="29" t="s">
-        <v>52</v>
-      </c>
-      <c r="B31" s="29"/>
-      <c r="C31" s="29"/>
-      <c r="D31" s="29"/>
-    </row>
-    <row r="32" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="s">
+    <row r="30" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="31" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="B31" s="20"/>
+      <c r="C31" s="27" t="n">
+        <f aca="false">SUM(C23:C29)</f>
+        <v>3130</v>
+      </c>
+      <c r="D31" s="22"/>
+    </row>
+    <row r="32" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="28" t="s">
+        <v>57</v>
+      </c>
+      <c r="B32" s="28"/>
+      <c r="C32" s="28"/>
+      <c r="D32" s="28"/>
+    </row>
+    <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="34" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="B34" s="29"/>
+      <c r="C34" s="29"/>
+      <c r="D34" s="29"/>
+    </row>
+    <row r="35" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B32" s="30" t="s">
-        <v>53</v>
-      </c>
-      <c r="C32" s="30"/>
-      <c r="D32" s="30"/>
-    </row>
-    <row r="33" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="B33" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="C33" s="11"/>
-      <c r="D33" s="11"/>
-    </row>
-    <row r="34" customFormat="false" ht="104.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="B34" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="C34" s="7"/>
-      <c r="D34" s="7"/>
-    </row>
-    <row r="35" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="B35" s="11" t="s">
+      <c r="B35" s="30" t="s">
         <v>59</v>
       </c>
-      <c r="C35" s="11"/>
-      <c r="D35" s="11"/>
+      <c r="C35" s="30"/>
+      <c r="D35" s="30"/>
     </row>
     <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
@@ -1298,7 +1328,7 @@
       <c r="C36" s="7"/>
       <c r="D36" s="7"/>
     </row>
-    <row r="37" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="104.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
         <v>62</v>
       </c>
@@ -1338,7 +1368,7 @@
       <c r="C40" s="7"/>
       <c r="D40" s="7"/>
     </row>
-    <row r="41" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="10" t="s">
         <v>70</v>
       </c>
@@ -1357,6 +1387,36 @@
       </c>
       <c r="C42" s="7"/>
       <c r="D42" s="7"/>
+    </row>
+    <row r="43" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="B43" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="C43" s="11"/>
+      <c r="D43" s="11"/>
+    </row>
+    <row r="44" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B44" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="C44" s="7"/>
+      <c r="D44" s="7"/>
+    </row>
+    <row r="45" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="B45" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="C45" s="11"/>
+      <c r="D45" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="19">
@@ -1365,12 +1425,9 @@
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="A21:D21"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A29:D29"/>
-    <mergeCell ref="A31:D31"/>
-    <mergeCell ref="B32:D32"/>
-    <mergeCell ref="B33:D33"/>
-    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="A34:D34"/>
     <mergeCell ref="B35:D35"/>
     <mergeCell ref="B36:D36"/>
     <mergeCell ref="B37:D37"/>
@@ -1379,6 +1436,9 @@
     <mergeCell ref="B40:D40"/>
     <mergeCell ref="B41:D41"/>
     <mergeCell ref="B42:D42"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="B45:D45"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
   <pageMargins left="0.3" right="0.3" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1389,7 +1449,7 @@
   </headerFooter>
   <rowBreaks count="2" manualBreakCount="2">
     <brk id="19" man="true" max="16383" min="0"/>
-    <brk id="29" man="true" max="16383" min="0"/>
+    <brk id="32" man="true" max="16383" min="0"/>
   </rowBreaks>
 </worksheet>
 </file>
</xml_diff>